<commit_message>
Add decision policy to lesson 1 agent
</commit_message>
<xml_diff>
--- a/generated_datasets/russia_languages_dataset_inventory.xlsx
+++ b/generated_datasets/russia_languages_dataset_inventory.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA43"/>
+  <dimension ref="A1:AE43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,6 +565,26 @@
           <t>checked_at_utc</t>
         </is>
       </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>agent_decision</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>agent_confidence</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>agent_next_actions</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>agent_review_reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -678,6 +698,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -791,6 +831,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -888,6 +948,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1001,6 +1081,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1114,6 +1214,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1227,6 +1347,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1340,6 +1480,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1453,6 +1613,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1566,6 +1746,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1679,6 +1879,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1792,6 +2012,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1897,6 +2137,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2002,6 +2262,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2115,6 +2395,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2228,6 +2528,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2341,6 +2661,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2454,6 +2794,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2567,6 +2927,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2680,6 +3060,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2793,6 +3193,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2906,6 +3326,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3019,6 +3459,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3132,6 +3592,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3237,6 +3717,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3350,6 +3850,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3463,6 +3983,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3576,6 +4116,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3689,6 +4249,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3802,6 +4382,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>accept_with_spot_check</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3915,6 +4515,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4028,6 +4648,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4141,6 +4781,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4254,6 +4914,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4359,6 +5039,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4464,6 +5164,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4569,6 +5289,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4666,6 +5406,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4763,6 +5523,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4860,6 +5640,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4957,6 +5757,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5062,6 +5882,26 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5157,6 +5997,26 @@
       <c r="AA43" t="inlineStr">
         <is>
           <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
         </is>
       </c>
     </row>
@@ -5171,7 +6031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5213,22 +6073,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>checked_at_utc</t>
+          <t>decision_policy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>Agent assigns accept_with_spot_check / needs_human_review / needs_discovery and next actions from OPUS/HF observations.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>checked_at_utc</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>caveat</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Counts are API snapshots and need linguistic/community review before publication.</t>
         </is>

</xml_diff>

<commit_message>
Convert lesson 1 notebook to dataset pipeline
</commit_message>
<xml_diff>
--- a/generated_datasets/russia_languages_dataset_inventory.xlsx
+++ b/generated_datasets/russia_languages_dataset_inventory.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE43"/>
+  <dimension ref="A1:AA43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,26 +565,6 @@
           <t>checked_at_utc</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>agent_decision</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>agent_confidence</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>agent_next_actions</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>agent_review_reason</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -671,7 +651,7 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>490277</v>
+        <v>493832</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -695,27 +675,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -804,11 +764,11 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>489569</v>
+        <v>492177</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K</t>
+          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K; n&gt;1T</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -828,27 +788,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -921,7 +861,7 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>161335</v>
+        <v>167099</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -945,27 +885,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1046,15 +966,15 @@
         <v>10</v>
       </c>
       <c r="T5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly; graelo/wikipedia</t>
+          <t>wikimedia/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; graelo/wikipedia; Helsinki-NLP/tatoeba</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>376897</v>
+        <v>382532</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -1078,27 +998,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1183,11 +1083,11 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly</t>
+          <t>anzorq/kbd-ru; wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>490104</v>
+        <v>492734</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1211,27 +1111,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1200,7 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>488902</v>
+        <v>491696</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1344,27 +1224,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1453,11 +1313,11 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>427866</v>
+        <v>542752</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; 1K&lt;n&lt;10K; 1M&lt;n&lt;10M</t>
+          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; 1K&lt;n&lt;10K; 1M&lt;n&lt;10M; n&lt;1K</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -1477,27 +1337,7 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1426,7 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>518780</v>
+        <v>522377</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1610,27 +1450,7 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1531,7 @@
         <v>11</v>
       </c>
       <c r="T10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1719,11 +1539,11 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>148788</v>
+        <v>168559</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K</t>
+          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -1743,27 +1563,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1848,11 +1648,11 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly</t>
+          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; graelo/wikipedia</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>487592</v>
+        <v>491349</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -1876,27 +1676,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1765,7 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>490254</v>
+        <v>493804</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -2009,27 +1789,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2106,11 +1866,11 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>mahesh27/archi_rutul_asr; openbmb/DCAD-2000; cointegrated/panlex-meanings; gtak1/panlex-meanings; AlidarAsvarov/dagestan-constitution</t>
+          <t>mahesh27/archi_rutul_asr; openbmb/DCAD-2000; cointegrated/panlex-meanings; gtak1/panlex-meanings; jake-anto/wiktionary</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>19453</v>
+        <v>19476</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -2134,27 +1894,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2235,7 +1975,7 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>19183</v>
+        <v>19137</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
@@ -2259,27 +1999,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE14" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2088,7 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>20476</v>
+        <v>20466</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
@@ -2392,27 +2112,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE15" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2201,7 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>410796</v>
+        <v>417248</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
@@ -2525,27 +2225,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE16" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2630,15 +2310,15 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly</t>
+          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; graelo/wikipedia</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>491422</v>
+        <v>494028</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K</t>
+          <t>100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K; n&gt;1T</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -2658,27 +2338,7 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2427,7 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>154663</v>
+        <v>160631</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
@@ -2791,27 +2451,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD18" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE18" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2540,7 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>144096</v>
+        <v>150158</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
@@ -2924,27 +2564,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3033,11 +2653,11 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>449265</v>
+        <v>472563</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; 1K&lt;n&lt;10K; 1M&lt;n&lt;10M; n&lt;1K</t>
+          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; 1K&lt;n&lt;10K; 1M&lt;n&lt;10M</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -3057,27 +2677,7 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB20" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE20" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3166,7 +2766,7 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>385214</v>
+        <v>391317</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
@@ -3190,27 +2790,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB21" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE21" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3299,7 +2879,7 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>146636</v>
+        <v>152549</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
@@ -3323,27 +2903,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB22" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC22" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE22" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3424,15 +2984,15 @@
         <v>10</v>
       </c>
       <c r="T23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly; graelo/wikipedia</t>
+          <t>wikimedia/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; cis-lmu/Glot500; graelo/wikipedia</t>
         </is>
       </c>
       <c r="V23" t="n">
-        <v>375915</v>
+        <v>384503</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
@@ -3456,27 +3016,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE23" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3561,11 +3101,11 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly</t>
+          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; graelo/wikipedia</t>
         </is>
       </c>
       <c r="V24" t="n">
-        <v>489544</v>
+        <v>494380</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
@@ -3589,27 +3129,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB24" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC24" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE24" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3202,7 @@
         <v>15</v>
       </c>
       <c r="T25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -3690,7 +3210,7 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>135195</v>
+        <v>143532</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
@@ -3714,27 +3234,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB25" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC25" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD25" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE25" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3823,11 +3323,11 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>414687</v>
+        <v>433329</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K</t>
+          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -3847,27 +3347,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE26" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3956,11 +3436,11 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>500207</v>
+        <v>502999</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K</t>
+          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K; n&gt;1T</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -3980,27 +3460,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB27" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC27" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD27" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE27" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4089,11 +3549,11 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>387125</v>
+        <v>394669</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>100B&lt;n&lt;1T; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B; n&lt;1K</t>
+          <t>100B&lt;n&lt;1T; 100K&lt;n&lt;1M; 100M&lt;n&lt;1B; 10K&lt;n&lt;100K; 10M&lt;n&lt;100M; 1B&lt;n&lt;10B</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
@@ -4113,27 +3573,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB28" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC28" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD28" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE28" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4222,7 +3662,7 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>500720</v>
+        <v>503672</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -4246,27 +3686,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB29" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC29" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD29" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE29" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4355,7 +3775,7 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>499114</v>
+        <v>504101</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
@@ -4379,27 +3799,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB30" t="inlineStr">
-        <is>
-          <t>accept_with_spot_check</t>
-        </is>
-      </c>
-      <c r="AC30" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="AD30" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE30" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4484,11 +3884,11 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; cointegrated/panlex-meanings; ayymen/Pontoon-Translations; Helsinki-NLP/tatoeba</t>
+          <t>HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; cointegrated/panlex-meanings; albertvillanova/universal_dependencies; ayymen/Pontoon-Translations</t>
         </is>
       </c>
       <c r="V31" t="n">
-        <v>135719</v>
+        <v>142402</v>
       </c>
       <c r="W31" t="inlineStr">
         <is>
@@ -4512,27 +3912,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC31" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD31" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE31" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4617,11 +3997,11 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; omarkamali/wikipedia-monthly</t>
+          <t>wikimedia/wikipedia; legacy-datasets/wikipedia; HuggingFaceFW/fineweb-2; HuggingFaceFW/finepdfs; graelo/wikipedia</t>
         </is>
       </c>
       <c r="V32" t="n">
-        <v>491147</v>
+        <v>493949</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
@@ -4645,27 +4025,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB32" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC32" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD32" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE32" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4750,11 +4110,11 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>udmurtNLP/flores-250-rus-udm; udmurtNLP/udmurt-russian-english-labse; udmurtNLP/soviet-geography-book-rus-udm-parallel-corpora; udmurtNLP/udmurt-bible-parallel-corpora; udmurtNLP/zerpal</t>
+          <t>udmurtNLP/flores-250-rus-udm; udmurtNLP/udmurt-russian-english-labse; udmurtNLP/soviet-geography-book-rus-udm-parallel-corpora; udmurtNLP/udmurt-bible-parallel-corpora; udmurtNLP/tatoeba-rus-udm-parallel-corpora</t>
         </is>
       </c>
       <c r="V33" t="n">
-        <v>491576</v>
+        <v>496765</v>
       </c>
       <c r="W33" t="inlineStr">
         <is>
@@ -4778,27 +4138,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB33" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC33" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD33" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE33" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4883,11 +4223,11 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>catherinearnett/veps; Lynxpda/original-veps-russian; Lynxpda/back-translated-russian-veps; Lynxpda/back-translated-veps-russian; Lynxpda/dic-veps-russian</t>
+          <t>catherinearnett/veps; Lynxpda/back-translated-russian-veps; Lynxpda/original-veps-russian; Lynxpda/dic-veps-russian; Lynxpda/back-translated-veps-russian</t>
         </is>
       </c>
       <c r="V34" t="n">
-        <v>394860</v>
+        <v>509686</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
@@ -4911,27 +4251,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC34" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD34" t="inlineStr">
-        <is>
-          <t>retry_opus_later; accept_opus_parallel_stats; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE34" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5012,7 +4332,7 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>138312</v>
+        <v>144897</v>
       </c>
       <c r="W35" t="inlineStr">
         <is>
@@ -5036,27 +4356,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB35" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC35" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD35" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE35" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5137,7 +4437,7 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>154488</v>
+        <v>160534</v>
       </c>
       <c r="W36" t="inlineStr">
         <is>
@@ -5161,27 +4461,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB36" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC36" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD36" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE36" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5262,7 +4542,7 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>140364</v>
+        <v>146440</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -5286,27 +4566,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB37" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC37" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD37" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE37" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5379,7 +4639,7 @@
         </is>
       </c>
       <c r="V38" t="n">
-        <v>142933</v>
+        <v>149023</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
@@ -5403,27 +4663,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB38" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC38" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD38" t="inlineStr">
-        <is>
-          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE38" t="inlineStr">
-        <is>
-          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5496,7 +4736,7 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>15493</v>
+        <v>15540</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
@@ -5520,27 +4760,7 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB39" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC39" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD39" t="inlineStr">
-        <is>
-          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE39" t="inlineStr">
-        <is>
-          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5613,7 +4833,7 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>14476</v>
+        <v>14548</v>
       </c>
       <c r="W40" t="inlineStr">
         <is>
@@ -5637,27 +4857,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB40" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC40" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD40" t="inlineStr">
-        <is>
-          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE40" t="inlineStr">
-        <is>
-          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5730,7 +4930,7 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>154211</v>
+        <v>160836</v>
       </c>
       <c r="W41" t="inlineStr">
         <is>
@@ -5754,27 +4954,7 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB41" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC41" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD41" t="inlineStr">
-        <is>
-          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE41" t="inlineStr">
-        <is>
-          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5855,7 +5035,7 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>9579</v>
+        <v>9455</v>
       </c>
       <c r="W42" t="inlineStr">
         <is>
@@ -5879,27 +5059,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB42" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC42" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD42" t="inlineStr">
-        <is>
-          <t>retry_opus_later; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE42" t="inlineStr">
-        <is>
-          <t>OPUS не ответил: статистика могла быть взята из кеша или остаться нулевой; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5132,7 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>151265</v>
+        <v>156829</v>
       </c>
       <c r="W43" t="inlineStr">
         <is>
@@ -5996,27 +5156,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="AB43" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="AC43" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AD43" t="inlineStr">
-        <is>
-          <t>review_language_code_mapping; search_parallel_candidates; inspect_hf_parallel_cards</t>
-        </is>
-      </c>
-      <c r="AE43" t="inlineStr">
-        <is>
-          <t>нет OPUS-кода: агент не может корректно проверить OPUS; OPUS не нашел русско-параллельные пары</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -6031,7 +5171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6073,34 +5213,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>decision_policy</t>
+          <t>checked_at_utc</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Agent assigns accept_with_spot_check / needs_human_review / needs_discovery and next actions from OPUS/HF observations.</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>checked_at_utc</t>
+          <t>caveat</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>caveat</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
         <is>
           <t>Counts are API snapshots and need linguistic/community review before publication.</t>
         </is>

</xml_diff>